<commit_message>
Health sector firms updated
</commit_message>
<xml_diff>
--- a/data/Health_sector_companies.xlsx
+++ b/data/Health_sector_companies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moham09/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moham09/Downloads/job-search-agent/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{312C21FA-E87C-8E4A-A58D-66BCC320A877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26909B9E-A538-AF46-90D7-08E07D5A6CDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{4BC829A6-0186-C14E-90CB-4600834BEDB2}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{4BC829A6-0186-C14E-90CB-4600834BEDB2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>#</t>
   </si>
@@ -110,6 +110,24 @@
   </si>
   <si>
     <t>https://jobs.lever.co/aledade</t>
+  </si>
+  <si>
+    <t>Globus Medical</t>
+  </si>
+  <si>
+    <t>https://globusmedical.wd5.myworkdayjobs.com/en-US/GMED_Careers</t>
+  </si>
+  <si>
+    <t>GE HealthCare</t>
+  </si>
+  <si>
+    <t>https://gehc.wd5.myworkdayjobs.com/GEHC_ExternalSite</t>
+  </si>
+  <si>
+    <t>Omnicell</t>
+  </si>
+  <si>
+    <t>https://apply.omnicell.com/careers/</t>
   </si>
 </sst>
 </file>
@@ -181,12 +199,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -502,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C21BC077-D33A-BA47-BE41-79152B5F9F54}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.33203125" customWidth="1"/>
@@ -522,7 +543,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" t="s">
@@ -533,7 +554,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3">
+      <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
@@ -544,7 +565,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" t="s">
@@ -555,7 +576,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5">
+      <c r="A5" s="3">
         <v>4</v>
       </c>
       <c r="B5" t="s">
@@ -566,7 +587,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6">
+      <c r="A6" s="3">
         <v>5</v>
       </c>
       <c r="B6" t="s">
@@ -577,7 +598,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7">
+      <c r="A7" s="3">
         <v>6</v>
       </c>
       <c r="B7" t="s">
@@ -588,7 +609,7 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8">
+      <c r="A8" s="3">
         <v>7</v>
       </c>
       <c r="B8" t="s">
@@ -599,7 +620,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9">
+      <c r="A9" s="3">
         <v>8</v>
       </c>
       <c r="B9" t="s">
@@ -610,7 +631,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10">
+      <c r="A10" s="3">
         <v>9</v>
       </c>
       <c r="B10" t="s">
@@ -621,7 +642,7 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11">
+      <c r="A11" s="3">
         <v>10</v>
       </c>
       <c r="B11" t="s">
@@ -632,7 +653,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12">
+      <c r="A12" s="3">
         <v>11</v>
       </c>
       <c r="B12" t="s">
@@ -640,6 +661,39 @@
       </c>
       <c r="C12" s="2" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -655,6 +709,9 @@
     <hyperlink ref="C10" r:id="rId9" xr:uid="{7CE41C9D-54AA-B748-AC9A-4EF1C31CC9B6}"/>
     <hyperlink ref="C11" r:id="rId10" xr:uid="{4181165B-EE2E-9E43-8A54-F14FF0370239}"/>
     <hyperlink ref="C12" r:id="rId11" xr:uid="{9426D8AB-A388-0443-B433-9D20D1569C79}"/>
+    <hyperlink ref="C13" r:id="rId12" xr:uid="{79839241-616E-CB4E-B889-34419BC9381E}"/>
+    <hyperlink ref="C14" r:id="rId13" xr:uid="{51D79506-9760-224B-8544-AAE9E02BADC4}"/>
+    <hyperlink ref="C15" r:id="rId14" xr:uid="{A411454C-FF35-5E45-AF86-F93D11A9E922}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>